<commit_message>
Redact SAP username from archived Metadata xlsx audit fields.
Replace ILIYAR with REDACTED in input/old Metadata exports so creator/editor names are not stored in the repo.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/input/old/Metadata _Bank account country differs from Vendor's country_SW_10_06_BNK_VND_COM_ARP.xlsx
+++ b/input/old/Metadata _Bank account country differs from Vendor's country_SW_10_06_BNK_VND_COM_ARP.xlsx
@@ -422,7 +422,7 @@
         <v>Created on</v>
       </c>
       <c r="B6" t="str">
-        <v>14.01.2026 at 16:17 by ILIYAR</v>
+        <v>14.01.2026 at 16:17 by REDACTED</v>
       </c>
     </row>
     <row r="7">
@@ -430,7 +430,7 @@
         <v>Updated on</v>
       </c>
       <c r="B7" t="str">
-        <v>14.01.2026 at 16:17 by ILIYAR</v>
+        <v>14.01.2026 at 16:17 by REDACTED</v>
       </c>
     </row>
     <row r="8">

</xml_diff>